<commit_message>
chore: update battle simulation data for bfmaster_1 and bfmaster_2 shield configurations with new Pokémon entries and performance metrics
</commit_message>
<xml_diff>
--- a/data/output/bfmaster.xlsx
+++ b/data/output/bfmaster.xlsx
@@ -36,48 +36,48 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>steel/ghost</t>
+          <t>steel/psychic</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Gengar (Mega) SC+ShP/SlB 15/15/15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>psychic/flying</t>
+          <t>ghost/poison</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Kyogre W+Av/OP 15/15/15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>dark/flying</t>
+          <t>water/none</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kyogre W+Av/OP 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>water/none</t>
+          <t>fairy/flying</t>
         </is>
       </c>
     </row>
@@ -96,12 +96,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>fairy/none</t>
+          <t>dragon/flying</t>
         </is>
       </c>
     </row>
@@ -171,7 +171,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -201,7 +201,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>191.3984748726641</v>
+        <v>166.55672080256633</v>
       </c>
     </row>
     <row r="10">
@@ -211,7 +211,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>152.3015873015873</v>
+        <v>78.3219814241486</v>
       </c>
     </row>
     <row r="11">
@@ -221,7 +221,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>208.14421800346267</v>
+        <v>160.65271462487303</v>
       </c>
     </row>
     <row r="12">
@@ -231,7 +231,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>768.6078431372549</v>
+        <v>823.2745098039217</v>
       </c>
     </row>
     <row r="13">
@@ -241,7 +241,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -251,7 +251,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>0.803921568627451</v>
+        <v>0.8627450980392157</v>
       </c>
     </row>
     <row r="15">
@@ -261,7 +261,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
@@ -271,7 +271,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>708.3137254901961</v>
+        <v>758.5686274509804</v>
       </c>
     </row>
     <row r="17">
@@ -281,7 +281,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -291,7 +291,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>0.0196078431372549</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="19">
@@ -321,7 +321,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22">
@@ -331,7 +331,7 @@
         </is>
       </c>
       <c r="B22">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23">
@@ -341,7 +341,7 @@
         </is>
       </c>
       <c r="B23">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
@@ -381,7 +381,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>87.6</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="28">
@@ -391,7 +391,7 @@
         </is>
       </c>
       <c r="B28">
-        <v>68.23333333333333</v>
+        <v>63.757746478873244</v>
       </c>
     </row>
     <row r="29">
@@ -401,7 +401,7 @@
         </is>
       </c>
       <c r="B29">
-        <v>54.4</v>
+        <v>28.9</v>
       </c>
     </row>
     <row r="30">
@@ -423,7 +423,7 @@
         </is>
       </c>
       <c r="B31">
-        <v>71.58333333333333</v>
+        <v>78.11666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="B32">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B33">
-        <v>0.058823529411764705</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="34">
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B35">
-        <v>630.9861111111112</v>
+        <v>715.5294117647059</v>
       </c>
     </row>
   </sheetData>
@@ -522,16 +522,16 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0.916667</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
@@ -596,7 +596,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -616,22 +616,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>ABA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+          <t>Kyogre W+Av/OP 15/15/15</t>
         </is>
       </c>
     </row>
@@ -646,17 +646,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Kyogre W+Av/OP 15/15/15</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
         </is>
       </c>
     </row>
@@ -671,17 +671,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Kyogre W+Av/OP 15/15/15</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
         </is>
       </c>
     </row>
@@ -696,17 +696,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Gengar (Mega) SC+ShP/SlB 15/15/15</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Kyogre W+Av/OP 15/15/15</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
         </is>
       </c>
     </row>
@@ -721,17 +721,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Gengar (Mega) SC+ShP/SlB 15/15/15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -751,12 +751,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -771,17 +771,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -796,17 +796,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -821,17 +821,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Kyogre W+Av/OP 15/15/15</t>
         </is>
       </c>
     </row>
@@ -867,36 +867,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Florges FW+TBl/CW 15/15/15</t>
+          <t>Swampert (Mega) MS+HC/Eq 15/15/15</t>
         </is>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0-shield only Gholdengo A+SB/FB 15/15/15 | 1-shield no cover</t>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Ampharos (Mega) VS+TBl/BrS 15/15/15</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Dialga (Origin) DB+ROT/IH 15/15/15</t>
         </is>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0-shield only Tyranitar DB+BrS/SE 15/15/15 | 1-shield only Zacian (Hero) Sn+WC/CC 15/15/15</t>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lugia (Shadow) DT+A/Fl 15/15/15</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Reshiram DB+FuF/SE 15/15/15</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dialga DB+IH/DM 15/15/15</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Zamazenta (Crowned Shield) IF+CC/BB 15/15/15</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gyarados (Shadow) DB+AT/Tw 15/15/15</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gholdengo A+SB/DG 15/15/15</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update battle simulation data for bfmaster_1 and bfmaster_2 shield configurations with new Pokémon entries and performance metrics (#5)
</commit_message>
<xml_diff>
--- a/data/output/bfmaster.xlsx
+++ b/data/output/bfmaster.xlsx
@@ -36,48 +36,48 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>steel/ghost</t>
+          <t>steel/psychic</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Gengar (Mega) SC+ShP/SlB 15/15/15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>psychic/flying</t>
+          <t>ghost/poison</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Kyogre W+Av/OP 15/15/15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>dark/flying</t>
+          <t>water/none</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kyogre W+Av/OP 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>water/none</t>
+          <t>fairy/flying</t>
         </is>
       </c>
     </row>
@@ -96,12 +96,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>fairy/none</t>
+          <t>dragon/flying</t>
         </is>
       </c>
     </row>
@@ -171,7 +171,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -201,7 +201,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>191.3984748726641</v>
+        <v>166.55672080256633</v>
       </c>
     </row>
     <row r="10">
@@ -211,7 +211,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>152.3015873015873</v>
+        <v>78.3219814241486</v>
       </c>
     </row>
     <row r="11">
@@ -221,7 +221,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>208.14421800346267</v>
+        <v>160.65271462487303</v>
       </c>
     </row>
     <row r="12">
@@ -231,7 +231,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>768.6078431372549</v>
+        <v>823.2745098039217</v>
       </c>
     </row>
     <row r="13">
@@ -241,7 +241,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -251,7 +251,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>0.803921568627451</v>
+        <v>0.8627450980392157</v>
       </c>
     </row>
     <row r="15">
@@ -261,7 +261,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
@@ -271,7 +271,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>708.3137254901961</v>
+        <v>758.5686274509804</v>
       </c>
     </row>
     <row r="17">
@@ -281,7 +281,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -291,7 +291,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>0.0196078431372549</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="19">
@@ -321,7 +321,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22">
@@ -331,7 +331,7 @@
         </is>
       </c>
       <c r="B22">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23">
@@ -341,7 +341,7 @@
         </is>
       </c>
       <c r="B23">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
@@ -381,7 +381,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>87.6</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="28">
@@ -391,7 +391,7 @@
         </is>
       </c>
       <c r="B28">
-        <v>68.23333333333333</v>
+        <v>63.757746478873244</v>
       </c>
     </row>
     <row r="29">
@@ -401,7 +401,7 @@
         </is>
       </c>
       <c r="B29">
-        <v>54.4</v>
+        <v>28.9</v>
       </c>
     </row>
     <row r="30">
@@ -423,7 +423,7 @@
         </is>
       </c>
       <c r="B31">
-        <v>71.58333333333333</v>
+        <v>78.11666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="B32">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B33">
-        <v>0.058823529411764705</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="34">
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B35">
-        <v>630.9861111111112</v>
+        <v>715.5294117647059</v>
       </c>
     </row>
   </sheetData>
@@ -522,16 +522,16 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0.916667</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
@@ -596,7 +596,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -616,22 +616,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>ABA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+          <t>Kyogre W+Av/OP 15/15/15</t>
         </is>
       </c>
     </row>
@@ -646,17 +646,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Kyogre W+Av/OP 15/15/15</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
         </is>
       </c>
     </row>
@@ -671,17 +671,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Kyogre W+Av/OP 15/15/15</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
         </is>
       </c>
     </row>
@@ -696,17 +696,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Gengar (Mega) SC+ShP/SlB 15/15/15</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Kyogre W+Av/OP 15/15/15</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
         </is>
       </c>
     </row>
@@ -721,17 +721,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Gengar (Mega) SC+ShP/SlB 15/15/15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -751,12 +751,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -771,17 +771,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tyranitar DB+BrS/SE 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -796,17 +796,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Togekiss Pk+DG/AuS 15/15/15</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Gholdengo A+SB/FB 15/15/15</t>
+          <t>Metagross SC+MM/Eq 15/15/15</t>
         </is>
       </c>
     </row>
@@ -821,17 +821,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lugia DT+A/Fl 15/15/15</t>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Zacian (Hero) Sn+WC/CC 15/15/15</t>
+          <t>Tyranitar DB+BrS/SE 15/15/15</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Yveltal SkP+DP/ObW 15/15/15</t>
+          <t>Kyogre W+Av/OP 15/15/15</t>
         </is>
       </c>
     </row>
@@ -867,36 +867,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Florges FW+TBl/CW 15/15/15</t>
+          <t>Swampert (Mega) MS+HC/Eq 15/15/15</t>
         </is>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0-shield only Gholdengo A+SB/FB 15/15/15 | 1-shield no cover</t>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Ampharos (Mega) VS+TBl/BrS 15/15/15</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dragonite DB+TP/SP 15/15/15</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Dialga (Origin) DB+ROT/IH 15/15/15</t>
         </is>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0-shield only Tyranitar DB+BrS/SE 15/15/15 | 1-shield only Zacian (Hero) Sn+WC/CC 15/15/15</t>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lugia (Shadow) DT+A/Fl 15/15/15</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Reshiram DB+FuF/SE 15/15/15</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dialga DB+IH/DM 15/15/15</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Zamazenta (Crowned Shield) IF+CC/BB 15/15/15</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gyarados (Shadow) DB+AT/Tw 15/15/15</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gholdengo A+SB/DG 15/15/15</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>

</xml_diff>